<commit_message>
Fixing COR and finished ROM plots, almost done yo
</commit_message>
<xml_diff>
--- a/New_CenterOfRotation/Finite_COR/Data Files/C45_Data/Model 1 Y_Z Data.xlsx
+++ b/New_CenterOfRotation/Finite_COR/Data Files/C45_Data/Model 1 Y_Z Data.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="2"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="4N"/>
@@ -2677,8 +2677,8 @@
       <c r="AC2" s="14"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="28" t="s">
-        <v>20</v>
+      <c r="A3" s="16" t="s">
+        <v>16</v>
       </c>
       <c r="B3" s="17">
         <v>25454</v>
@@ -2686,8 +2686,8 @@
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
       <c r="E3" s="10"/>
-      <c r="F3" s="28" t="s">
-        <v>20</v>
+      <c r="F3" s="16" t="s">
+        <v>16</v>
       </c>
       <c r="G3" s="17">
         <v>31067</v>
@@ -2695,8 +2695,8 @@
       <c r="H3" s="12"/>
       <c r="I3" s="12"/>
       <c r="J3" s="10"/>
-      <c r="K3" s="28" t="s">
-        <v>20</v>
+      <c r="K3" s="16" t="s">
+        <v>16</v>
       </c>
       <c r="L3" s="18">
         <v>29005</v>
@@ -2704,8 +2704,8 @@
       <c r="M3" s="19"/>
       <c r="N3" s="19"/>
       <c r="O3" s="10"/>
-      <c r="P3" s="28" t="s">
-        <v>20</v>
+      <c r="P3" s="16" t="s">
+        <v>16</v>
       </c>
       <c r="Q3" s="18">
         <v>45615</v>
@@ -2713,8 +2713,8 @@
       <c r="R3" s="19"/>
       <c r="S3" s="19"/>
       <c r="T3" s="10"/>
-      <c r="U3" s="28" t="s">
-        <v>20</v>
+      <c r="U3" s="16" t="s">
+        <v>16</v>
       </c>
       <c r="V3" s="18">
         <v>52027</v>
@@ -2722,8 +2722,8 @@
       <c r="W3" s="19"/>
       <c r="X3" s="19"/>
       <c r="Y3" s="10"/>
-      <c r="Z3" s="29" t="s">
-        <v>20</v>
+      <c r="Z3" s="20" t="s">
+        <v>17</v>
       </c>
       <c r="AA3" s="21">
         <v>49903</v>
@@ -4673,8 +4673,8 @@
       <c r="AC2" s="14"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="28" t="s">
-        <v>20</v>
+      <c r="A3" s="16" t="s">
+        <v>16</v>
       </c>
       <c r="B3" s="17">
         <v>25454</v>
@@ -4682,8 +4682,8 @@
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
       <c r="E3" s="10"/>
-      <c r="F3" s="28" t="s">
-        <v>20</v>
+      <c r="F3" s="16" t="s">
+        <v>16</v>
       </c>
       <c r="G3" s="17">
         <v>31067</v>
@@ -4691,8 +4691,8 @@
       <c r="H3" s="12"/>
       <c r="I3" s="12"/>
       <c r="J3" s="10"/>
-      <c r="K3" s="28" t="s">
-        <v>20</v>
+      <c r="K3" s="16" t="s">
+        <v>16</v>
       </c>
       <c r="L3" s="18">
         <v>29005</v>
@@ -4700,8 +4700,8 @@
       <c r="M3" s="19"/>
       <c r="N3" s="19"/>
       <c r="O3" s="10"/>
-      <c r="P3" s="28" t="s">
-        <v>20</v>
+      <c r="P3" s="16" t="s">
+        <v>16</v>
       </c>
       <c r="Q3" s="18">
         <v>45615</v>
@@ -4709,8 +4709,8 @@
       <c r="R3" s="19"/>
       <c r="S3" s="19"/>
       <c r="T3" s="10"/>
-      <c r="U3" s="28" t="s">
-        <v>20</v>
+      <c r="U3" s="16" t="s">
+        <v>16</v>
       </c>
       <c r="V3" s="18">
         <v>52027</v>
@@ -4718,8 +4718,8 @@
       <c r="W3" s="19"/>
       <c r="X3" s="19"/>
       <c r="Y3" s="10"/>
-      <c r="Z3" s="29" t="s">
-        <v>20</v>
+      <c r="Z3" s="20" t="s">
+        <v>17</v>
       </c>
       <c r="AA3" s="21">
         <v>49903</v>
@@ -6669,8 +6669,8 @@
       <c r="AC2" s="14"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="28" t="s">
-        <v>20</v>
+      <c r="A3" s="16" t="s">
+        <v>16</v>
       </c>
       <c r="B3" s="17">
         <v>25454</v>
@@ -6678,8 +6678,8 @@
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
       <c r="E3" s="10"/>
-      <c r="F3" s="28" t="s">
-        <v>20</v>
+      <c r="F3" s="16" t="s">
+        <v>16</v>
       </c>
       <c r="G3" s="17">
         <v>31067</v>
@@ -6687,8 +6687,8 @@
       <c r="H3" s="12"/>
       <c r="I3" s="12"/>
       <c r="J3" s="10"/>
-      <c r="K3" s="28" t="s">
-        <v>20</v>
+      <c r="K3" s="16" t="s">
+        <v>16</v>
       </c>
       <c r="L3" s="18">
         <v>29005</v>
@@ -6696,8 +6696,8 @@
       <c r="M3" s="19"/>
       <c r="N3" s="19"/>
       <c r="O3" s="10"/>
-      <c r="P3" s="28" t="s">
-        <v>20</v>
+      <c r="P3" s="16" t="s">
+        <v>16</v>
       </c>
       <c r="Q3" s="18">
         <v>45615</v>
@@ -6705,8 +6705,8 @@
       <c r="R3" s="19"/>
       <c r="S3" s="19"/>
       <c r="T3" s="10"/>
-      <c r="U3" s="28" t="s">
-        <v>20</v>
+      <c r="U3" s="16" t="s">
+        <v>16</v>
       </c>
       <c r="V3" s="18">
         <v>52027</v>
@@ -6714,8 +6714,8 @@
       <c r="W3" s="19"/>
       <c r="X3" s="19"/>
       <c r="Y3" s="10"/>
-      <c r="Z3" s="29" t="s">
-        <v>20</v>
+      <c r="Z3" s="20" t="s">
+        <v>17</v>
       </c>
       <c r="AA3" s="21">
         <v>49903</v>

</xml_diff>